<commit_message>
A avoid crash algorithm
</commit_message>
<xml_diff>
--- a/controllers/Nao_defender/改进表.xlsx
+++ b/controllers/Nao_defender/改进表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Mrobotic\TDP\Nao_test_keeperAndDefender\controllers\Nao_defender\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D8EA5BA-3743-49A5-B22C-AFF0D50C24A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC7E4460-16BE-4FDF-81D5-D3BE4ED85532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="5025" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>改进/修复</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -52,6 +52,18 @@
   </si>
   <si>
     <t>striker-球-自己 三点一线</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>类似AGVS向量式避碰导航</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2/10/2025</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>向量避碰下的vice模式debug</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -377,10 +389,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.25" customWidth="1"/>
+    <col min="1" max="1" width="22.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -403,14 +415,30 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>